<commit_message>
feat: enhance generate_seed_templates.ts with detailed product and service data
Updated seed template generator to include extensive product catalog with realistic specifications, pricing, categories, and service offerings. Removed hardcoded image arrays in favor of verified Unsplash and document URLs. Added support for both products and services with structured data including offers, bulk deals, and technical specifications to improve seeding realism and utility.
</commit_message>
<xml_diff>
--- a/backend/seeded_templates/Seeded_Products_Import.xlsx
+++ b/backend/seeded_templates/Seeded_Products_Import.xlsx
@@ -477,19 +477,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Premium Industrial Product Variant 1</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="B2" t="str">
-        <v>Fuel, Oil &amp; Gas</v>
+        <v>Steel &amp; Metal Products</v>
       </c>
       <c r="C2" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D2" t="str">
-        <v>High quality industrial product 1 with premium build. Ideal for heavy duty applications.</v>
+        <v>High-strength thermo-mechanically treated Fe 550D rebars with superior bendability, ductility, and seismic resistance for industrial RCC structures.</v>
       </c>
       <c r="E2">
-        <v>150</v>
+        <v>58500</v>
       </c>
       <c r="F2" t="str">
         <v>INR</v>
@@ -498,19 +498,19 @@
         <v>18</v>
       </c>
       <c r="H2" t="str">
-        <v>Nos</v>
+        <v>MT</v>
       </c>
       <c r="I2" t="str">
-        <v>HSN8001</v>
+        <v>721420</v>
       </c>
       <c r="J2" t="str">
-        <v>PROD-2026-1001</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="K2" t="str">
-        <v>IndustrialBrand1</v>
+        <v>Jindal Panther / Tata Tiscon</v>
       </c>
       <c r="L2" t="str">
-        <v>MOD-PRO-1</v>
+        <v>FE-550D-12MM</v>
       </c>
       <c r="M2" t="str">
         <v>NEW</v>
@@ -519,22 +519,22 @@
         <v>Yes</v>
       </c>
       <c r="O2">
-        <v>180</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
+        <v>62000</v>
+      </c>
+      <c r="P2">
+        <v>58500</v>
+      </c>
+      <c r="Q2">
+        <v>5.65</v>
       </c>
       <c r="R2" t="str">
-        <v>Special Offer</v>
+        <v>District Infrastructure Bulk Rate</v>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U2" t="str">
         <v>Yes</v>
@@ -543,27 +543,27 @@
         <v>10</v>
       </c>
       <c r="W2" t="str">
-        <v>https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122, https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092335397-9583eb92d232</v>
+        <v>https://images.unsplash.com/photo-1618090584176-7132b9911657?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X2" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Premium Industrial Product Variant 2</v>
+        <v>Industrial Safety Helmet Class-E with 6-Point Ratchet</v>
       </c>
       <c r="B3" t="str">
-        <v>Power &amp; Energy Equipment</v>
+        <v>Safety Equipment &amp; Industrial Safety</v>
       </c>
       <c r="C3" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D3" t="str">
-        <v>High quality industrial product 2 with premium build. Ideal for heavy duty applications.</v>
+        <v>High-density polyethylene (HDPE) electrical shock-proof safety helmet with 6-point nylon ratchet harness, chin strap, and sweatband.</v>
       </c>
       <c r="E3">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="F3" t="str">
         <v>INR</v>
@@ -575,16 +575,16 @@
         <v>Nos</v>
       </c>
       <c r="I3" t="str">
-        <v>HSN8002</v>
+        <v>650610</v>
       </c>
       <c r="J3" t="str">
-        <v>PROD-2026-1002</v>
+        <v>SAF-HLM-PRO-E</v>
       </c>
       <c r="K3" t="str">
-        <v>IndustrialBrand2</v>
+        <v>Karam / Udyogi</v>
       </c>
       <c r="L3" t="str">
-        <v>MOD-PRO-2</v>
+        <v>SHEL-E500</v>
       </c>
       <c r="M3" t="str">
         <v>NEW</v>
@@ -593,51 +593,51 @@
         <v>Yes</v>
       </c>
       <c r="O3">
-        <v>360</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
+        <v>550</v>
+      </c>
+      <c r="P3">
+        <v>450</v>
+      </c>
+      <c r="Q3">
+        <v>18.18</v>
       </c>
       <c r="R3" t="str">
-        <v>Special Offer</v>
+        <v>MSME Site Safety Special</v>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U3" t="str">
         <v>Yes</v>
       </c>
       <c r="V3">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W3" t="str">
-        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952</v>
+        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X3" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Premium Industrial Product Variant 3</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="B4" t="str">
-        <v>Refractories</v>
+        <v>Pipes, Tiles &amp; Hardware</v>
       </c>
       <c r="C4" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D4" t="str">
-        <v>High quality industrial product 3 with premium build. Ideal for heavy duty applications.</v>
+        <v>Cast carbon steel two-piece full bore flanged ball valve designed for industrial steam, oil, water, and gas isolation pipelines.</v>
       </c>
       <c r="E4">
-        <v>450</v>
+        <v>9200</v>
       </c>
       <c r="F4" t="str">
         <v>INR</v>
@@ -649,16 +649,16 @@
         <v>Nos</v>
       </c>
       <c r="I4" t="str">
-        <v>HSN8003</v>
+        <v>848180</v>
       </c>
       <c r="J4" t="str">
-        <v>PROD-2026-1003</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="K4" t="str">
-        <v>IndustrialBrand3</v>
+        <v>Audco / L&amp;T</v>
       </c>
       <c r="L4" t="str">
-        <v>MOD-PRO-3</v>
+        <v>FB-CS300-4IN</v>
       </c>
       <c r="M4" t="str">
         <v>NEW</v>
@@ -667,51 +667,51 @@
         <v>Yes</v>
       </c>
       <c r="O4">
-        <v>540</v>
-      </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
-        <v/>
+        <v>10500</v>
+      </c>
+      <c r="P4">
+        <v>9200</v>
+      </c>
+      <c r="Q4">
+        <v>12.38</v>
       </c>
       <c r="R4" t="str">
-        <v>Special Offer</v>
+        <v>Plant Spares Special</v>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U4" t="str">
         <v>Yes</v>
       </c>
       <c r="V4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="W4" t="str">
-        <v>https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122</v>
+        <v>https://images.unsplash.com/photo-1565043666747-69f6646db940?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X4" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Premium Industrial Product Variant 4</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="B5" t="str">
-        <v>Automobile Parts &amp; Services</v>
+        <v>Pumps, Motors &amp; Hydraulics</v>
       </c>
       <c r="C5" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D5" t="str">
-        <v>High quality industrial product 4 with premium build. Ideal for heavy duty applications.</v>
+        <v>Energy-efficient IE3 cast iron frame 3-phase induction motor with IP55 protection for severe industrial environments and continuous duty S1.</v>
       </c>
       <c r="E5">
-        <v>600</v>
+        <v>36800</v>
       </c>
       <c r="F5" t="str">
         <v>INR</v>
@@ -723,16 +723,16 @@
         <v>Nos</v>
       </c>
       <c r="I5" t="str">
-        <v>HSN8004</v>
+        <v>850152</v>
       </c>
       <c r="J5" t="str">
-        <v>PROD-2026-1004</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="K5" t="str">
-        <v>IndustrialBrand4</v>
+        <v>Bharat Bijlee / ABB</v>
       </c>
       <c r="L5" t="str">
-        <v>MOD-PRO-4</v>
+        <v>IE3-160M-4P</v>
       </c>
       <c r="M5" t="str">
         <v>NEW</v>
@@ -741,51 +741,51 @@
         <v>Yes</v>
       </c>
       <c r="O5">
-        <v>720</v>
-      </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
-        <v/>
+        <v>42000</v>
+      </c>
+      <c r="P5">
+        <v>36800</v>
+      </c>
+      <c r="Q5">
+        <v>12.38</v>
       </c>
       <c r="R5" t="str">
-        <v>Special Offer</v>
+        <v>Factory Modernization Offer</v>
       </c>
       <c r="S5" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T5" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U5" t="str">
         <v>Yes</v>
       </c>
       <c r="V5">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W5" t="str">
-        <v>https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158</v>
+        <v>https://images.unsplash.com/photo-1581092160607-ee22621dd758?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X5" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Premium Industrial Product Variant 5</v>
+        <v>1.1 kV XLPE 4-Core Aluminium Armoured Power Cable (185 sq.mm)</v>
       </c>
       <c r="B6" t="str">
-        <v>Office Equipment &amp; Stationery</v>
+        <v>Electrical Cables &amp; Power Equipment</v>
       </c>
       <c r="C6" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D6" t="str">
-        <v>High quality industrial product 5 with premium build. Ideal for heavy duty applications.</v>
+        <v>Heavy duty stranded aluminium conductor underground armoured power cable with cross-linked polyethylene (XLPE) insulation and galvanized steel strip armour.</v>
       </c>
       <c r="E6">
-        <v>750</v>
+        <v>1150</v>
       </c>
       <c r="F6" t="str">
         <v>INR</v>
@@ -794,19 +794,19 @@
         <v>18</v>
       </c>
       <c r="H6" t="str">
-        <v>Nos</v>
+        <v>Meter</v>
       </c>
       <c r="I6" t="str">
-        <v>HSN8005</v>
+        <v>854449</v>
       </c>
       <c r="J6" t="str">
-        <v>PROD-2026-1005</v>
+        <v>CBL-PWR-4C-185AL</v>
       </c>
       <c r="K6" t="str">
-        <v>IndustrialBrand5</v>
+        <v>Polycab / Havells</v>
       </c>
       <c r="L6" t="str">
-        <v>MOD-PRO-5</v>
+        <v>A2XFY-4X185</v>
       </c>
       <c r="M6" t="str">
         <v>NEW</v>
@@ -815,51 +815,51 @@
         <v>Yes</v>
       </c>
       <c r="O6">
-        <v>900</v>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v/>
+        <v>1280</v>
+      </c>
+      <c r="P6">
+        <v>1150</v>
+      </c>
+      <c r="Q6">
+        <v>10.16</v>
       </c>
       <c r="R6" t="str">
-        <v>Special Offer</v>
+        <v>Substation Project Rate</v>
       </c>
       <c r="S6" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T6" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U6" t="str">
         <v>Yes</v>
       </c>
       <c r="V6">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="W6" t="str">
-        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1530124566582-a618bc2615dc</v>
+        <v>https://images.unsplash.com/photo-1621905251189-08b45d6a269e?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X6" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Premium Industrial Product Variant 6</v>
+        <v>Grade 8.8 High-Tensile Hot-Dip Galvanized Hex Bolts &amp; Nuts (M16 x 80mm)</v>
       </c>
       <c r="B7" t="str">
-        <v>Bearings &amp; Mechanical Components</v>
+        <v>Industrial Fasteners &amp; Components</v>
       </c>
       <c r="C7" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D7" t="str">
-        <v>High quality industrial product 6 with premium build. Ideal for heavy duty applications.</v>
+        <v>Precision forged high-tensile structural bolts conforming to DIN 933 with matching heavy hex nuts and spring washers, hot-dip galvanized for corrosion resistance.</v>
       </c>
       <c r="E7">
-        <v>900</v>
+        <v>48</v>
       </c>
       <c r="F7" t="str">
         <v>INR</v>
@@ -871,16 +871,16 @@
         <v>Nos</v>
       </c>
       <c r="I7" t="str">
-        <v>HSN8006</v>
+        <v>731815</v>
       </c>
       <c r="J7" t="str">
-        <v>PROD-2026-1006</v>
+        <v>FAS-HEX-M16-80</v>
       </c>
       <c r="K7" t="str">
-        <v>IndustrialBrand6</v>
+        <v>Sundram Fasteners / Unbrako</v>
       </c>
       <c r="L7" t="str">
-        <v>MOD-PRO-6</v>
+        <v>HDG-8.8-M16</v>
       </c>
       <c r="M7" t="str">
         <v>NEW</v>
@@ -889,51 +889,51 @@
         <v>Yes</v>
       </c>
       <c r="O7">
-        <v>1080</v>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-      <c r="Q7" t="str">
-        <v/>
+        <v>55</v>
+      </c>
+      <c r="P7">
+        <v>48</v>
+      </c>
+      <c r="Q7">
+        <v>12.73</v>
       </c>
       <c r="R7" t="str">
-        <v>Special Offer</v>
+        <v>Bulk Erection Fasteners Deal</v>
       </c>
       <c r="S7" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T7" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U7" t="str">
         <v>Yes</v>
       </c>
       <c r="V7">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="W7" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158</v>
+        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X7" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Premium Industrial Product Variant 7</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="B8" t="str">
-        <v>Construction &amp; Building Materials</v>
+        <v>Bearings &amp; Mechanical Components</v>
       </c>
       <c r="C8" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D8" t="str">
-        <v>High quality industrial product 7 with premium build. Ideal for heavy duty applications.</v>
+        <v>Single row deep groove ball bearing with C3 radial internal clearance and dual synthetic rubber contact seals on both sides for heavy industrial vibration duties.</v>
       </c>
       <c r="E8">
-        <v>1050</v>
+        <v>1850</v>
       </c>
       <c r="F8" t="str">
         <v>INR</v>
@@ -945,16 +945,16 @@
         <v>Nos</v>
       </c>
       <c r="I8" t="str">
-        <v>HSN8007</v>
+        <v>848210</v>
       </c>
       <c r="J8" t="str">
-        <v>PROD-2026-1007</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="K8" t="str">
-        <v>IndustrialBrand7</v>
+        <v>SKF / FAG</v>
       </c>
       <c r="L8" t="str">
-        <v>MOD-PRO-7</v>
+        <v>6312-2RS1-C3</v>
       </c>
       <c r="M8" t="str">
         <v>NEW</v>
@@ -963,22 +963,22 @@
         <v>Yes</v>
       </c>
       <c r="O8">
-        <v>1260</v>
-      </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-      <c r="Q8" t="str">
-        <v/>
+        <v>2100</v>
+      </c>
+      <c r="P8">
+        <v>1850</v>
+      </c>
+      <c r="Q8">
+        <v>11.9</v>
       </c>
       <c r="R8" t="str">
-        <v>Special Offer</v>
+        <v>Original Spares Assured</v>
       </c>
       <c r="S8" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T8" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U8" t="str">
         <v>Yes</v>
@@ -987,27 +987,27 @@
         <v>10</v>
       </c>
       <c r="W8" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1530124566582-a618bc2615dc</v>
+        <v>https://images.unsplash.com/photo-1581092334651-ddf26d9a09d0?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X8" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Premium Industrial Product Variant 8</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="B9" t="str">
-        <v>Steel &amp; Metal Products</v>
+        <v>Hydraulics &amp; Pneumatics</v>
       </c>
       <c r="C9" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D9" t="str">
-        <v>High quality industrial product 8 with premium build. Ideal for heavy duty applications.</v>
+        <v>Tie-rod industrial hydraulic ram cylinder engineered for 210 bar working pressure with hard chrome plated rod and imported polyurethane chevron seals.</v>
       </c>
       <c r="E9">
-        <v>1200</v>
+        <v>26500</v>
       </c>
       <c r="F9" t="str">
         <v>INR</v>
@@ -1019,16 +1019,16 @@
         <v>Nos</v>
       </c>
       <c r="I9" t="str">
-        <v>HSN8008</v>
+        <v>841221</v>
       </c>
       <c r="J9" t="str">
-        <v>PROD-2026-1008</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="K9" t="str">
-        <v>IndustrialBrand8</v>
+        <v>Yuken / Rexroth MSME Partner</v>
       </c>
       <c r="L9" t="str">
-        <v>MOD-PRO-8</v>
+        <v>HC-210B-100-400</v>
       </c>
       <c r="M9" t="str">
         <v>NEW</v>
@@ -1037,72 +1037,72 @@
         <v>Yes</v>
       </c>
       <c r="O9">
-        <v>1440</v>
-      </c>
-      <c r="P9" t="str">
-        <v/>
-      </c>
-      <c r="Q9" t="str">
-        <v/>
+        <v>31000</v>
+      </c>
+      <c r="P9">
+        <v>26500</v>
+      </c>
+      <c r="Q9">
+        <v>14.52</v>
       </c>
       <c r="R9" t="str">
-        <v>Special Offer</v>
+        <v>Hydraulics Manufacturer Special</v>
       </c>
       <c r="S9" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T9" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U9" t="str">
         <v>Yes</v>
       </c>
       <c r="V9">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W9" t="str">
-        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158</v>
+        <v>https://images.unsplash.com/photo-1581092162384-8987c1d64718?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X9" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Premium Industrial Product Variant 9</v>
+        <v>Portland Slag Cement (PSC) 50 Kg Moisture-Proof Bags</v>
       </c>
       <c r="B10" t="str">
-        <v>FMCG &amp; Daily Utility Supply</v>
+        <v>Cement &amp; Concrete Products</v>
       </c>
       <c r="C10" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D10" t="str">
-        <v>High quality industrial product 9 with premium build. Ideal for heavy duty applications.</v>
+        <v>High performance slag cement manufactured with high glass content granulated blast furnace slag. Exceptional resistance to chemical and sulphate attack.</v>
       </c>
       <c r="E10">
-        <v>1350</v>
+        <v>345</v>
       </c>
       <c r="F10" t="str">
         <v>INR</v>
       </c>
       <c r="G10">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H10" t="str">
-        <v>Nos</v>
+        <v>Bags</v>
       </c>
       <c r="I10" t="str">
-        <v>HSN8009</v>
+        <v>252329</v>
       </c>
       <c r="J10" t="str">
-        <v>PROD-2026-1009</v>
+        <v>CEM-PSC-50KG</v>
       </c>
       <c r="K10" t="str">
-        <v>IndustrialBrand9</v>
+        <v>UltraTech / Dalmia</v>
       </c>
       <c r="L10" t="str">
-        <v>MOD-PRO-9</v>
+        <v>PSC-IS455</v>
       </c>
       <c r="M10" t="str">
         <v>NEW</v>
@@ -1111,51 +1111,51 @@
         <v>Yes</v>
       </c>
       <c r="O10">
-        <v>1620</v>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
-        <v/>
+        <v>380</v>
+      </c>
+      <c r="P10">
+        <v>345</v>
+      </c>
+      <c r="Q10">
+        <v>9.21</v>
       </c>
       <c r="R10" t="str">
-        <v>Special Offer</v>
+        <v>Construction Bulk Depot Price</v>
       </c>
       <c r="S10" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T10" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U10" t="str">
         <v>Yes</v>
       </c>
       <c r="V10">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="W10" t="str">
-        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122, https://images.unsplash.com/photo-1581092335397-9583eb92d232</v>
+        <v>https://images.unsplash.com/photo-1587293852726-70cdb56c2866?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X10" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Premium Industrial Product Variant 10</v>
+        <v>IGBT Multi-Process Inverter Welding Machine (400 Amp, 3-Phase)</v>
       </c>
       <c r="B11" t="str">
-        <v>teeeeeee</v>
+        <v>Welding &amp; Cutting Equipment</v>
       </c>
       <c r="C11" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D11" t="str">
-        <v>High quality industrial product 10 with premium build. Ideal for heavy duty applications.</v>
+        <v>Heavy duty digital industrial MMA/TIG inverter arc welding machine with thermal overload protection, arc force adjustment, and anti-stick features.</v>
       </c>
       <c r="E11">
-        <v>1500</v>
+        <v>32000</v>
       </c>
       <c r="F11" t="str">
         <v>INR</v>
@@ -1167,16 +1167,16 @@
         <v>Nos</v>
       </c>
       <c r="I11" t="str">
-        <v>HSN8010</v>
+        <v>851539</v>
       </c>
       <c r="J11" t="str">
-        <v>PROD-2026-1010</v>
+        <v>WELD-INV-400A-3P</v>
       </c>
       <c r="K11" t="str">
-        <v>IndustrialBrand10</v>
+        <v>ESAB / Ador Welding</v>
       </c>
       <c r="L11" t="str">
-        <v>MOD-PRO-10</v>
+        <v>ARC-400-IGBT</v>
       </c>
       <c r="M11" t="str">
         <v>NEW</v>
@@ -1185,51 +1185,51 @@
         <v>Yes</v>
       </c>
       <c r="O11">
-        <v>1800</v>
-      </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-      <c r="Q11" t="str">
-        <v/>
+        <v>37500</v>
+      </c>
+      <c r="P11">
+        <v>32000</v>
+      </c>
+      <c r="Q11">
+        <v>14.67</v>
       </c>
       <c r="R11" t="str">
-        <v>Special Offer</v>
+        <v>Fabrication Workshop Kit</v>
       </c>
       <c r="S11" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T11" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U11" t="str">
         <v>Yes</v>
       </c>
       <c r="V11">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W11" t="str">
-        <v>https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1530124566582-a618bc2615dc</v>
+        <v>https://images.unsplash.com/photo-1581092583537-20d51b4b4f1b?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X11" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Premium Industrial Product Variant 11</v>
+        <v>High Alumina 70% Industrial Refractory Fire Bricks (IS 8 Standard)</v>
       </c>
       <c r="B12" t="str">
-        <v>Industrial Chemicals</v>
+        <v>Refractories</v>
       </c>
       <c r="C12" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D12" t="str">
-        <v>High quality industrial product 11 with premium build. Ideal for heavy duty applications.</v>
+        <v>High-density Al2O3 refractory bricks for blast furnaces, steel reheating furnaces, rotary kilns, and high-temperature thermal power incinerators.</v>
       </c>
       <c r="E12">
-        <v>1650</v>
+        <v>72</v>
       </c>
       <c r="F12" t="str">
         <v>INR</v>
@@ -1241,16 +1241,16 @@
         <v>Nos</v>
       </c>
       <c r="I12" t="str">
-        <v>HSN8011</v>
+        <v>690220</v>
       </c>
       <c r="J12" t="str">
-        <v>PROD-2026-1011</v>
+        <v>REF-BRK-HA70-IS8</v>
       </c>
       <c r="K12" t="str">
-        <v>IndustrialBrand11</v>
+        <v>TRL Krosaki / RHI Magnesita</v>
       </c>
       <c r="L12" t="str">
-        <v>MOD-PRO-11</v>
+        <v>HA-70-STD</v>
       </c>
       <c r="M12" t="str">
         <v>NEW</v>
@@ -1259,72 +1259,72 @@
         <v>Yes</v>
       </c>
       <c r="O12">
-        <v>1980</v>
-      </c>
-      <c r="P12" t="str">
-        <v/>
-      </c>
-      <c r="Q12" t="str">
-        <v/>
+        <v>85</v>
+      </c>
+      <c r="P12">
+        <v>72</v>
+      </c>
+      <c r="Q12">
+        <v>15.29</v>
       </c>
       <c r="R12" t="str">
-        <v>Special Offer</v>
+        <v>Thermal Kiln Maintenance Special</v>
       </c>
       <c r="S12" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U12" t="str">
         <v>Yes</v>
       </c>
       <c r="V12">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="W12" t="str">
-        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952</v>
+        <v>https://images.unsplash.com/photo-1587293852726-70cdb56c2866?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X12" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Premium Industrial Product Variant 12</v>
+        <v>Authentic Sambalpuri Handloom Pure Cotton Ikat Saree (GI Certified)</v>
       </c>
       <c r="B13" t="str">
-        <v>Electrical Cables &amp; Power Equipment</v>
+        <v>Textile &amp; Garments Supply</v>
       </c>
       <c r="C13" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D13" t="str">
-        <v>High quality industrial product 12 with premium build. Ideal for heavy duty applications.</v>
+        <v>Traditional handcrafted Sambalpuri cotton saree produced by registered Odisha SHG weavers with intricate tie-and-dye Ikat floral border and pallu.</v>
       </c>
       <c r="E13">
-        <v>1800</v>
+        <v>3400</v>
       </c>
       <c r="F13" t="str">
         <v>INR</v>
       </c>
       <c r="G13">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H13" t="str">
         <v>Nos</v>
       </c>
       <c r="I13" t="str">
-        <v>HSN8012</v>
+        <v>520852</v>
       </c>
       <c r="J13" t="str">
-        <v>PROD-2026-1012</v>
+        <v>SHG-SAM-SAREE-01</v>
       </c>
       <c r="K13" t="str">
-        <v>IndustrialBrand12</v>
+        <v>Boyanika / Odisha Weavers Federation</v>
       </c>
       <c r="L13" t="str">
-        <v>MOD-PRO-12</v>
+        <v>SAM-IKAT-100C</v>
       </c>
       <c r="M13" t="str">
         <v>NEW</v>
@@ -1333,22 +1333,22 @@
         <v>Yes</v>
       </c>
       <c r="O13">
-        <v>2160</v>
-      </c>
-      <c r="P13" t="str">
-        <v/>
-      </c>
-      <c r="Q13" t="str">
-        <v/>
+        <v>4200</v>
+      </c>
+      <c r="P13">
+        <v>3400</v>
+      </c>
+      <c r="Q13">
+        <v>19.05</v>
       </c>
       <c r="R13" t="str">
-        <v>Special Offer</v>
+        <v>herSHG Artisan Direct Fair</v>
       </c>
       <c r="S13" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T13" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U13" t="str">
         <v>Yes</v>
@@ -1357,24 +1357,24 @@
         <v>10</v>
       </c>
       <c r="W13" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1530124566582-a618bc2615dc</v>
+        <v>https://images.unsplash.com/photo-1610030469983-98e550d6193c?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X13" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Premium Industrial Product Variant 13</v>
+        <v>Odisha Dhokra Brass Lost-Wax Casting Tribal Art Figurine (8-Inch)</v>
       </c>
       <c r="B14" t="str">
-        <v>Industrial Consumables</v>
+        <v>FMCG &amp; Daily Utility Supply</v>
       </c>
       <c r="C14" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D14" t="str">
-        <v>High quality industrial product 13 with premium build. Ideal for heavy duty applications.</v>
+        <v>Handmade bell-metal non-ferrous casting made by tribal artisan self-help groups using ancient lost-wax technique. Ideal for corporate gifts &amp; mementos.</v>
       </c>
       <c r="E14">
         <v>1950</v>
@@ -1383,22 +1383,22 @@
         <v>INR</v>
       </c>
       <c r="G14">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H14" t="str">
         <v>Nos</v>
       </c>
       <c r="I14" t="str">
-        <v>HSN8013</v>
+        <v>830629</v>
       </c>
       <c r="J14" t="str">
-        <v>PROD-2026-1013</v>
+        <v>SHG-DHK-FIG-08</v>
       </c>
       <c r="K14" t="str">
-        <v>IndustrialBrand13</v>
+        <v>Utkalika / Tribal SHG Federation</v>
       </c>
       <c r="L14" t="str">
-        <v>MOD-PRO-13</v>
+        <v>DHOKRA-8IN</v>
       </c>
       <c r="M14" t="str">
         <v>NEW</v>
@@ -1407,51 +1407,51 @@
         <v>Yes</v>
       </c>
       <c r="O14">
-        <v>2340</v>
-      </c>
-      <c r="P14" t="str">
-        <v/>
-      </c>
-      <c r="Q14" t="str">
-        <v/>
+        <v>2400</v>
+      </c>
+      <c r="P14">
+        <v>1950</v>
+      </c>
+      <c r="Q14">
+        <v>18.75</v>
       </c>
       <c r="R14" t="str">
-        <v>Special Offer</v>
+        <v>Tribal Handicrafts Promotion</v>
       </c>
       <c r="S14" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T14" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U14" t="str">
         <v>Yes</v>
       </c>
       <c r="V14">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="W14" t="str">
-        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158</v>
+        <v>https://images.unsplash.com/photo-1590736704728-f4730bb30770?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X14" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Premium Industrial Product Variant 14</v>
+        <v>Industrial Heavy Duty Nitrile Chemical Gauntlet Gloves (15-Inch, 15 Mil)</v>
       </c>
       <c r="B15" t="str">
-        <v>IT &amp; Computer Equipment</v>
+        <v>Safety Equipment &amp; Industrial Safety</v>
       </c>
       <c r="C15" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D15" t="str">
-        <v>High quality industrial product 14 with premium build. Ideal for heavy duty applications.</v>
+        <v>Flock-lined green nitrile gloves offering premium resistance against corrosive acids, caustic solvents, oils, and grease in chemical plants and refineries.</v>
       </c>
       <c r="E15">
-        <v>2100</v>
+        <v>240</v>
       </c>
       <c r="F15" t="str">
         <v>INR</v>
@@ -1460,19 +1460,19 @@
         <v>18</v>
       </c>
       <c r="H15" t="str">
-        <v>Nos</v>
+        <v>Pair</v>
       </c>
       <c r="I15" t="str">
-        <v>HSN8014</v>
+        <v>401519</v>
       </c>
       <c r="J15" t="str">
-        <v>PROD-2026-1014</v>
+        <v>SAF-GLV-NIT-15</v>
       </c>
       <c r="K15" t="str">
-        <v>IndustrialBrand14</v>
+        <v>Ansell / Honeywell</v>
       </c>
       <c r="L15" t="str">
-        <v>MOD-PRO-14</v>
+        <v>SOLVEX-15M</v>
       </c>
       <c r="M15" t="str">
         <v>NEW</v>
@@ -1481,51 +1481,51 @@
         <v>Yes</v>
       </c>
       <c r="O15">
-        <v>2520</v>
-      </c>
-      <c r="P15" t="str">
-        <v/>
-      </c>
-      <c r="Q15" t="str">
-        <v/>
+        <v>290</v>
+      </c>
+      <c r="P15">
+        <v>240</v>
+      </c>
+      <c r="Q15">
+        <v>17.24</v>
       </c>
       <c r="R15" t="str">
-        <v>Special Offer</v>
+        <v>PPE Bulk Deal</v>
       </c>
       <c r="S15" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T15" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U15" t="str">
         <v>Yes</v>
       </c>
       <c r="V15">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="W15" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581092335397-9583eb92d232</v>
+        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X15" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Premium Industrial Product Variant 15</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="B16" t="str">
-        <v>Tools &amp; Industrial Hardware</v>
+        <v>Conveyor &amp; Material Handling Equipment</v>
       </c>
       <c r="C16" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D16" t="str">
-        <v>High quality industrial product 15 with premium build. Ideal for heavy duty applications.</v>
+        <v>Heavy duty multi-ply rubber conveyor belting with polyester warp and polyamide weft fabric for transporting coal, clinker, limestone, and ore.</v>
       </c>
       <c r="E16">
-        <v>2250</v>
+        <v>2600</v>
       </c>
       <c r="F16" t="str">
         <v>INR</v>
@@ -1534,19 +1534,19 @@
         <v>18</v>
       </c>
       <c r="H16" t="str">
-        <v>Nos</v>
+        <v>Meter</v>
       </c>
       <c r="I16" t="str">
-        <v>HSN8015</v>
+        <v>401012</v>
       </c>
       <c r="J16" t="str">
-        <v>PROD-2026-1015</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="K16" t="str">
-        <v>IndustrialBrand15</v>
+        <v>Dunlop / Fenner</v>
       </c>
       <c r="L16" t="str">
-        <v>MOD-PRO-15</v>
+        <v>EP400-3PLY-HR</v>
       </c>
       <c r="M16" t="str">
         <v>NEW</v>
@@ -1555,51 +1555,51 @@
         <v>Yes</v>
       </c>
       <c r="O16">
-        <v>2700</v>
-      </c>
-      <c r="P16" t="str">
-        <v/>
-      </c>
-      <c r="Q16" t="str">
-        <v/>
+        <v>3000</v>
+      </c>
+      <c r="P16">
+        <v>2600</v>
+      </c>
+      <c r="Q16">
+        <v>13.33</v>
       </c>
       <c r="R16" t="str">
-        <v>Special Offer</v>
+        <v>Bulk Mining Conveyor Discount</v>
       </c>
       <c r="S16" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U16" t="str">
         <v>Yes</v>
       </c>
       <c r="V16">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W16" t="str">
-        <v>https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122</v>
+        <v>https://images.unsplash.com/photo-1586528116311-ad8dd3c8310d?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X16" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Premium Industrial Product Variant 16</v>
+        <v>Technical Grade Caustic Soda Flakes / Sodium Hydroxide (99.5% Pure, 50kg)</v>
       </c>
       <c r="B17" t="str">
-        <v>Furniture &amp; Interior Supplies</v>
+        <v>Industrial Chemicals</v>
       </c>
       <c r="C17" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D17" t="str">
-        <v>High quality industrial product 16 with premium build. Ideal for heavy duty applications.</v>
+        <v>High-purity sodium hydroxide flakes used extensively in alumina refining, water treatment, paper manufacturing, and textile effluent neutralization.</v>
       </c>
       <c r="E17">
-        <v>2400</v>
+        <v>2850</v>
       </c>
       <c r="F17" t="str">
         <v>INR</v>
@@ -1608,19 +1608,19 @@
         <v>18</v>
       </c>
       <c r="H17" t="str">
-        <v>Nos</v>
+        <v>Bags</v>
       </c>
       <c r="I17" t="str">
-        <v>HSN8016</v>
+        <v>281511</v>
       </c>
       <c r="J17" t="str">
-        <v>PROD-2026-1016</v>
+        <v>CHM-CS-FLK-50KG</v>
       </c>
       <c r="K17" t="str">
-        <v>IndustrialBrand16</v>
+        <v>GACL / DCM Shriram</v>
       </c>
       <c r="L17" t="str">
-        <v>MOD-PRO-16</v>
+        <v>NaOH-99.5-FLK</v>
       </c>
       <c r="M17" t="str">
         <v>NEW</v>
@@ -1629,72 +1629,72 @@
         <v>Yes</v>
       </c>
       <c r="O17">
-        <v>2880</v>
-      </c>
-      <c r="P17" t="str">
-        <v/>
-      </c>
-      <c r="Q17" t="str">
-        <v/>
+        <v>3200</v>
+      </c>
+      <c r="P17">
+        <v>2850</v>
+      </c>
+      <c r="Q17">
+        <v>10.94</v>
       </c>
       <c r="R17" t="str">
-        <v>Special Offer</v>
+        <v>Chemical Bulk Tanker / Bagged Deal</v>
       </c>
       <c r="S17" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T17" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U17" t="str">
         <v>Yes</v>
       </c>
       <c r="V17">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="W17" t="str">
-        <v>https://images.unsplash.com/photo-1581091226825-a6a2a5aee158, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122</v>
+        <v>https://images.unsplash.com/photo-1587293852726-70cdb56c2866?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X17" t="str">
-        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Premium Industrial Product Variant 17</v>
+        <v>Heavy Duty Mining Dumper Radial Tyre (10.00 R20 16PR All-Steel)</v>
       </c>
       <c r="B18" t="str">
-        <v>General Industrial Supplier</v>
+        <v>Tyres &amp; Rubber Products</v>
       </c>
       <c r="C18" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D18" t="str">
-        <v>High quality industrial product 17 with premium build. Ideal for heavy duty applications.</v>
+        <v>All-steel radial commercial truck and dumper tyre engineered with stone-ejecting grooves and chip-resistant tread compound for rough quarry mining roads.</v>
       </c>
       <c r="E18">
-        <v>2550</v>
+        <v>22800</v>
       </c>
       <c r="F18" t="str">
         <v>INR</v>
       </c>
       <c r="G18">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H18" t="str">
         <v>Nos</v>
       </c>
       <c r="I18" t="str">
-        <v>HSN8017</v>
+        <v>401120</v>
       </c>
       <c r="J18" t="str">
-        <v>PROD-2026-1017</v>
+        <v>TYR-R20-16PR-HD</v>
       </c>
       <c r="K18" t="str">
-        <v>IndustrialBrand17</v>
+        <v>Apollo / MRF / BKT</v>
       </c>
       <c r="L18" t="str">
-        <v>MOD-PRO-17</v>
+        <v>LUG-PLUS-1000R20</v>
       </c>
       <c r="M18" t="str">
         <v>NEW</v>
@@ -1703,51 +1703,51 @@
         <v>Yes</v>
       </c>
       <c r="O18">
-        <v>3060</v>
-      </c>
-      <c r="P18" t="str">
-        <v/>
-      </c>
-      <c r="Q18" t="str">
-        <v/>
+        <v>25500</v>
+      </c>
+      <c r="P18">
+        <v>22800</v>
+      </c>
+      <c r="Q18">
+        <v>10.59</v>
       </c>
       <c r="R18" t="str">
-        <v>Special Offer</v>
+        <v>Mining Fleet Maintenance Price</v>
       </c>
       <c r="S18" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T18" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U18" t="str">
         <v>Yes</v>
       </c>
       <c r="V18">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="W18" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581092335397-9583eb92d232</v>
+        <v>https://images.unsplash.com/photo-1517524008697-84bbe3c3fd98?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X18" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Premium Industrial Product Variant 18</v>
+        <v>Enterprise 2U Rackmount Server Dual Intel Xeon Silver 64GB ECC RAM</v>
       </c>
       <c r="B19" t="str">
-        <v>Gas Equipment &amp; Cylinders</v>
+        <v>IT &amp; Computer Equipment</v>
       </c>
       <c r="C19" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D19" t="str">
-        <v>High quality industrial product 18 with premium build. Ideal for heavy duty applications.</v>
+        <v>Mission-critical enterprise rack server configured with dual scalable Intel Xeon processors, redundant 80-Plus Platinum power supplies, and RAID controller.</v>
       </c>
       <c r="E19">
-        <v>2700</v>
+        <v>195000</v>
       </c>
       <c r="F19" t="str">
         <v>INR</v>
@@ -1759,69 +1759,69 @@
         <v>Nos</v>
       </c>
       <c r="I19" t="str">
-        <v>HSN8018</v>
+        <v>847150</v>
       </c>
       <c r="J19" t="str">
-        <v>PROD-2026-1018</v>
+        <v>IT-SRV-2U-XEON-64</v>
       </c>
       <c r="K19" t="str">
-        <v>IndustrialBrand18</v>
+        <v>Dell PowerEdge / HP ProLiant</v>
       </c>
       <c r="L19" t="str">
-        <v>MOD-PRO-18</v>
+        <v>PE-R750-XEON</v>
       </c>
       <c r="M19" t="str">
         <v>NEW</v>
       </c>
       <c r="N19" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="O19">
-        <v>3240</v>
-      </c>
-      <c r="P19" t="str">
-        <v/>
-      </c>
-      <c r="Q19" t="str">
-        <v/>
+        <v>220000</v>
+      </c>
+      <c r="P19">
+        <v>195000</v>
+      </c>
+      <c r="Q19">
+        <v>11.36</v>
       </c>
       <c r="R19" t="str">
-        <v>Special Offer</v>
+        <v>Enterprise Digital Infrastructure Special</v>
       </c>
       <c r="S19" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T19" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U19" t="str">
         <v>Yes</v>
       </c>
       <c r="V19">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="W19" t="str">
-        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122</v>
+        <v>https://images.unsplash.com/photo-1558494949-ef010cbdcc31?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X19" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Premium Industrial Product Variant 19</v>
+        <v>Pneumatic Heavy Duty Industrial Air Impact Wrench (1-Inch Drive, 2600 Nm)</v>
       </c>
       <c r="B20" t="str">
-        <v>Agriculture &amp; Nursery</v>
+        <v>Tools &amp; Industrial Hardware</v>
       </c>
       <c r="C20" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D20" t="str">
-        <v>High quality industrial product 19 with premium build. Ideal for heavy duty applications.</v>
+        <v>Pin-less hammer mechanism air impact wrench delivering up to 2600 Nm break-away torque for heavy truck wheel lug nuts and heavy structural bolting.</v>
       </c>
       <c r="E20">
-        <v>2850</v>
+        <v>19500</v>
       </c>
       <c r="F20" t="str">
         <v>INR</v>
@@ -1833,16 +1833,16 @@
         <v>Nos</v>
       </c>
       <c r="I20" t="str">
-        <v>HSN8019</v>
+        <v>846711</v>
       </c>
       <c r="J20" t="str">
-        <v>PROD-2026-1019</v>
+        <v>TOOL-AIW-1IN-2600</v>
       </c>
       <c r="K20" t="str">
-        <v>IndustrialBrand19</v>
+        <v>Ingersoll Rand / Chicago Pneumatic</v>
       </c>
       <c r="L20" t="str">
-        <v>MOD-PRO-19</v>
+        <v>IR-2600-1IN</v>
       </c>
       <c r="M20" t="str">
         <v>NEW</v>
@@ -1851,51 +1851,51 @@
         <v>Yes</v>
       </c>
       <c r="O20">
-        <v>3420</v>
-      </c>
-      <c r="P20" t="str">
-        <v/>
-      </c>
-      <c r="Q20" t="str">
-        <v/>
+        <v>23000</v>
+      </c>
+      <c r="P20">
+        <v>19500</v>
+      </c>
+      <c r="Q20">
+        <v>15.22</v>
       </c>
       <c r="R20" t="str">
-        <v>Special Offer</v>
+        <v>Workshop Tooling Bundle</v>
       </c>
       <c r="S20" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T20" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U20" t="str">
         <v>Yes</v>
       </c>
       <c r="V20">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="W20" t="str">
-        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc, https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1504917595217-d4dc5ebe6122</v>
+        <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X20" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/xfa_xobject.pdf</v>
+        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Premium Industrial Product Variant 20</v>
+        <v>Industrial PLC Automation Control Panel with 7-Inch Color Touch HMI</v>
       </c>
       <c r="B21" t="str">
-        <v>Industrial Seals &amp; Gaskets</v>
+        <v>Automation &amp; Robotics</v>
       </c>
       <c r="C21" t="str">
         <v>ACTIVE</v>
       </c>
       <c r="D21" t="str">
-        <v>High quality industrial product 20 with premium build. Ideal for heavy duty applications.</v>
+        <v>Custom-built IP65 electrical automation control desk panel incorporating programmable logic controller, variable frequency drives, SMPS, and safety relays.</v>
       </c>
       <c r="E21">
-        <v>3000</v>
+        <v>98000</v>
       </c>
       <c r="F21" t="str">
         <v>INR</v>
@@ -1904,19 +1904,19 @@
         <v>18</v>
       </c>
       <c r="H21" t="str">
-        <v>Nos</v>
+        <v>Set</v>
       </c>
       <c r="I21" t="str">
-        <v>HSN8020</v>
+        <v>853710</v>
       </c>
       <c r="J21" t="str">
-        <v>PROD-2026-1020</v>
+        <v>AUTO-PLC-PNL-7HMI</v>
       </c>
       <c r="K21" t="str">
-        <v>IndustrialBrand20</v>
+        <v>Siemens / Schneider MSME Integrator</v>
       </c>
       <c r="L21" t="str">
-        <v>MOD-PRO-20</v>
+        <v>S7-1200-HMI7</v>
       </c>
       <c r="M21" t="str">
         <v>NEW</v>
@@ -1925,34 +1925,34 @@
         <v>Yes</v>
       </c>
       <c r="O21">
-        <v>3600</v>
-      </c>
-      <c r="P21" t="str">
-        <v/>
-      </c>
-      <c r="Q21" t="str">
-        <v/>
+        <v>115000</v>
+      </c>
+      <c r="P21">
+        <v>98000</v>
+      </c>
+      <c r="Q21">
+        <v>14.78</v>
       </c>
       <c r="R21" t="str">
-        <v>Special Offer</v>
+        <v>Industrial Automation Promotion</v>
       </c>
       <c r="S21" t="str">
-        <v/>
+        <v>2026-09-01</v>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>2026-12-31</v>
       </c>
       <c r="U21" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="V21">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="W21" t="str">
-        <v>https://images.unsplash.com/photo-1581092335397-9583eb92d232, https://images.unsplash.com/photo-1581092160562-40aa08e11576, https://images.unsplash.com/photo-1581092795360-fd1ca04f0952, https://images.unsplash.com/photo-1581091226825-a6a2a5aee158</v>
+        <v>https://images.unsplash.com/photo-1581092580497-e0d23cbdf1dc?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X21" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf, https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
       </c>
     </row>
   </sheetData>
@@ -1964,7 +1964,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E88"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1985,16 +1985,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>PROD-2026-1001</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="B2" t="str">
-        <v>Premium Industrial Product Variant 1</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="C2" t="str">
-        <v>Material</v>
+        <v>Grade</v>
       </c>
       <c r="D2" t="str">
-        <v>High-Grade Alloy Type 1</v>
+        <v>Fe 550D</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -2002,33 +2002,33 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PROD-2026-1001</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="B3" t="str">
-        <v>Premium Industrial Product Variant 1</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="C3" t="str">
-        <v>Weight</v>
+        <v>Diameter</v>
       </c>
       <c r="D3" t="str">
-        <v>1.5</v>
+        <v>12</v>
       </c>
       <c r="E3" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PROD-2026-1001</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="B4" t="str">
-        <v>Premium Industrial Product Variant 1</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="C4" t="str">
-        <v>Warranty</v>
+        <v>Standard</v>
       </c>
       <c r="D4" t="str">
-        <v>2 Years</v>
+        <v>IS 1786:2008</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -2036,84 +2036,84 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>PROD-2026-1001</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="B5" t="str">
-        <v>Premium Industrial Product Variant 1</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="C5" t="str">
-        <v>Safety Standard</v>
+        <v>Yield Strength</v>
       </c>
       <c r="D5" t="str">
-        <v>ISO 9001:2015</v>
+        <v>550</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>N/mm²</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PROD-2026-1002</v>
+        <v>STEEL-TMT-550D-12</v>
       </c>
       <c r="B6" t="str">
-        <v>Premium Industrial Product Variant 2</v>
+        <v>Fe 550D TMT Rebar (12mm x 12m Bundles)</v>
       </c>
       <c r="C6" t="str">
-        <v>Material</v>
+        <v>Elongation</v>
       </c>
       <c r="D6" t="str">
-        <v>High-Grade Alloy Type 2</v>
+        <v>14.5</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>%</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>PROD-2026-1002</v>
+        <v>SAF-HLM-PRO-E</v>
       </c>
       <c r="B7" t="str">
-        <v>Premium Industrial Product Variant 2</v>
+        <v>Industrial Safety Helmet Class-E with 6-Point Ratchet</v>
       </c>
       <c r="C7" t="str">
-        <v>Weight</v>
+        <v>Shell Material</v>
       </c>
       <c r="D7" t="str">
-        <v>3</v>
+        <v>High-Density Polyethylene (HDPE)</v>
       </c>
       <c r="E7" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>PROD-2026-1002</v>
+        <v>SAF-HLM-PRO-E</v>
       </c>
       <c r="B8" t="str">
-        <v>Premium Industrial Product Variant 2</v>
+        <v>Industrial Safety Helmet Class-E with 6-Point Ratchet</v>
       </c>
       <c r="C8" t="str">
-        <v>Warranty</v>
+        <v>Electrical Resistance</v>
       </c>
       <c r="D8" t="str">
-        <v>2 Years</v>
+        <v>20000</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>Volts</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PROD-2026-1002</v>
+        <v>SAF-HLM-PRO-E</v>
       </c>
       <c r="B9" t="str">
-        <v>Premium Industrial Product Variant 2</v>
+        <v>Industrial Safety Helmet Class-E with 6-Point Ratchet</v>
       </c>
       <c r="C9" t="str">
-        <v>Safety Standard</v>
+        <v>Standard Certification</v>
       </c>
       <c r="D9" t="str">
-        <v>ISO 9001:2015</v>
+        <v>IS 2925:1984 / EN 397</v>
       </c>
       <c r="E9" t="str">
         <v/>
@@ -2121,67 +2121,67 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>PROD-2026-1003</v>
+        <v>SAF-HLM-PRO-E</v>
       </c>
       <c r="B10" t="str">
-        <v>Premium Industrial Product Variant 3</v>
+        <v>Industrial Safety Helmet Class-E with 6-Point Ratchet</v>
       </c>
       <c r="C10" t="str">
-        <v>Material</v>
+        <v>Impact Energy Absorption</v>
       </c>
       <c r="D10" t="str">
-        <v>High-Grade Alloy Type 3</v>
+        <v>50</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Joules</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>PROD-2026-1003</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="B11" t="str">
-        <v>Premium Industrial Product Variant 3</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="C11" t="str">
-        <v>Weight</v>
+        <v>Body Material</v>
       </c>
       <c r="D11" t="str">
-        <v>4.5</v>
+        <v>ASTM A216 Gr. WCB</v>
       </c>
       <c r="E11" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>PROD-2026-1003</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="B12" t="str">
-        <v>Premium Industrial Product Variant 3</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="C12" t="str">
-        <v>Warranty</v>
+        <v>Nominal Size</v>
       </c>
       <c r="D12" t="str">
-        <v>2 Years</v>
+        <v>4</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>Inch</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>PROD-2026-1003</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="B13" t="str">
-        <v>Premium Industrial Product Variant 3</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="C13" t="str">
-        <v>Safety Standard</v>
+        <v>Pressure Rating</v>
       </c>
       <c r="D13" t="str">
-        <v>ISO 9001:2015</v>
+        <v>Class 300 (PN 50)</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2189,16 +2189,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>PROD-2026-1004</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="B14" t="str">
-        <v>Premium Industrial Product Variant 4</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="C14" t="str">
-        <v>Material</v>
+        <v>End Connection</v>
       </c>
       <c r="D14" t="str">
-        <v>High-Grade Alloy Type 4</v>
+        <v>Flanged RF (ASME B16.5)</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -2206,101 +2206,101 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>PROD-2026-1004</v>
+        <v>VALV-BV-CS-100</v>
       </c>
       <c r="B15" t="str">
-        <v>Premium Industrial Product Variant 4</v>
+        <v>High-Pressure Carbon Steel Flanged Ball Valve (Class 300, 4-Inch)</v>
       </c>
       <c r="C15" t="str">
-        <v>Weight</v>
+        <v>Hydrostatic Shell Test</v>
       </c>
       <c r="D15" t="str">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="E15" t="str">
-        <v>Kg</v>
+        <v>Bar</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>PROD-2026-1004</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B16" t="str">
-        <v>Premium Industrial Product Variant 4</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C16" t="str">
-        <v>Warranty</v>
+        <v>Rated Output</v>
       </c>
       <c r="D16" t="str">
-        <v>2 Years</v>
+        <v>11</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>kW</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>PROD-2026-1004</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B17" t="str">
-        <v>Premium Industrial Product Variant 4</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C17" t="str">
-        <v>Safety Standard</v>
+        <v>Horsepower</v>
       </c>
       <c r="D17" t="str">
-        <v>ISO 9001:2015</v>
+        <v>15</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>HP</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>PROD-2026-1005</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B18" t="str">
-        <v>Premium Industrial Product Variant 5</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C18" t="str">
-        <v>Material</v>
+        <v>Speed</v>
       </c>
       <c r="D18" t="str">
-        <v>High-Grade Alloy Type 5</v>
+        <v>1440</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>RPM</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PROD-2026-1005</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B19" t="str">
-        <v>Premium Industrial Product Variant 5</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C19" t="str">
-        <v>Weight</v>
+        <v>Efficiency Class</v>
       </c>
       <c r="D19" t="str">
-        <v>7.5</v>
+        <v>IE3 Premium Efficiency</v>
       </c>
       <c r="E19" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>PROD-2026-1005</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B20" t="str">
-        <v>Premium Industrial Product Variant 5</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C20" t="str">
-        <v>Warranty</v>
+        <v>Frame Size</v>
       </c>
       <c r="D20" t="str">
-        <v>2 Years</v>
+        <v>160M</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -2308,16 +2308,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>PROD-2026-1005</v>
+        <v>MOT-IND-15HP-4P</v>
       </c>
       <c r="B21" t="str">
-        <v>Premium Industrial Product Variant 5</v>
+        <v>3-Phase Squirrel Cage Induction Motor (15 HP / 11 kW, 1440 RPM)</v>
       </c>
       <c r="C21" t="str">
-        <v>Safety Standard</v>
+        <v>Enclosure / IP Rating</v>
       </c>
       <c r="D21" t="str">
-        <v>ISO 9001:2015</v>
+        <v>IP55 Totally Enclosed Fan Cooled</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -2325,50 +2325,50 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>PROD-2026-1006</v>
+        <v>CBL-PWR-4C-185AL</v>
       </c>
       <c r="B22" t="str">
-        <v>Premium Industrial Product Variant 6</v>
+        <v>1.1 kV XLPE 4-Core Aluminium Armoured Power Cable (185 sq.mm)</v>
       </c>
       <c r="C22" t="str">
-        <v>Material</v>
+        <v>Voltage Rating</v>
       </c>
       <c r="D22" t="str">
-        <v>High-Grade Alloy Type 6</v>
+        <v>1100</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>V</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>PROD-2026-1006</v>
+        <v>CBL-PWR-4C-185AL</v>
       </c>
       <c r="B23" t="str">
-        <v>Premium Industrial Product Variant 6</v>
+        <v>1.1 kV XLPE 4-Core Aluminium Armoured Power Cable (185 sq.mm)</v>
       </c>
       <c r="C23" t="str">
-        <v>Weight</v>
+        <v>Cross Sectional Area</v>
       </c>
       <c r="D23" t="str">
-        <v>9</v>
+        <v>185</v>
       </c>
       <c r="E23" t="str">
-        <v>Kg</v>
+        <v>sq.mm</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>PROD-2026-1006</v>
+        <v>CBL-PWR-4C-185AL</v>
       </c>
       <c r="B24" t="str">
-        <v>Premium Industrial Product Variant 6</v>
+        <v>1.1 kV XLPE 4-Core Aluminium Armoured Power Cable (185 sq.mm)</v>
       </c>
       <c r="C24" t="str">
-        <v>Warranty</v>
+        <v>Conductor Material</v>
       </c>
       <c r="D24" t="str">
-        <v>2 Years</v>
+        <v>EC Grade Stranded Aluminium</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -2376,16 +2376,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>PROD-2026-1006</v>
+        <v>CBL-PWR-4C-185AL</v>
       </c>
       <c r="B25" t="str">
-        <v>Premium Industrial Product Variant 6</v>
+        <v>1.1 kV XLPE 4-Core Aluminium Armoured Power Cable (185 sq.mm)</v>
       </c>
       <c r="C25" t="str">
-        <v>Safety Standard</v>
+        <v>Standard</v>
       </c>
       <c r="D25" t="str">
-        <v>ISO 9001:2015</v>
+        <v>IS 7098 (Part 1)</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -2393,16 +2393,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>PROD-2026-1007</v>
+        <v>FAS-HEX-M16-80</v>
       </c>
       <c r="B26" t="str">
-        <v>Premium Industrial Product Variant 7</v>
+        <v>Grade 8.8 High-Tensile Hot-Dip Galvanized Hex Bolts &amp; Nuts (M16 x 80mm)</v>
       </c>
       <c r="C26" t="str">
-        <v>Material</v>
+        <v>Thread Size</v>
       </c>
       <c r="D26" t="str">
-        <v>High-Grade Alloy Type 7</v>
+        <v>M16 x 2.0mm</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -2410,33 +2410,33 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>PROD-2026-1007</v>
+        <v>FAS-HEX-M16-80</v>
       </c>
       <c r="B27" t="str">
-        <v>Premium Industrial Product Variant 7</v>
+        <v>Grade 8.8 High-Tensile Hot-Dip Galvanized Hex Bolts &amp; Nuts (M16 x 80mm)</v>
       </c>
       <c r="C27" t="str">
-        <v>Weight</v>
+        <v>Bolt Length</v>
       </c>
       <c r="D27" t="str">
-        <v>10.5</v>
+        <v>80</v>
       </c>
       <c r="E27" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>PROD-2026-1007</v>
+        <v>FAS-HEX-M16-80</v>
       </c>
       <c r="B28" t="str">
-        <v>Premium Industrial Product Variant 7</v>
+        <v>Grade 8.8 High-Tensile Hot-Dip Galvanized Hex Bolts &amp; Nuts (M16 x 80mm)</v>
       </c>
       <c r="C28" t="str">
-        <v>Warranty</v>
+        <v>Property Class</v>
       </c>
       <c r="D28" t="str">
-        <v>2 Years</v>
+        <v>8.8</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -2444,16 +2444,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>PROD-2026-1007</v>
+        <v>FAS-HEX-M16-80</v>
       </c>
       <c r="B29" t="str">
-        <v>Premium Industrial Product Variant 7</v>
+        <v>Grade 8.8 High-Tensile Hot-Dip Galvanized Hex Bolts &amp; Nuts (M16 x 80mm)</v>
       </c>
       <c r="C29" t="str">
-        <v>Safety Standard</v>
+        <v>Coating</v>
       </c>
       <c r="D29" t="str">
-        <v>ISO 9001:2015</v>
+        <v>Hot Dip Galvanized (HDG &gt; 45 micron)</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -2461,186 +2461,186 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PROD-2026-1008</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="B30" t="str">
-        <v>Premium Industrial Product Variant 8</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="C30" t="str">
-        <v>Material</v>
+        <v>Bore Diameter (d)</v>
       </c>
       <c r="D30" t="str">
-        <v>High-Grade Alloy Type 8</v>
+        <v>60</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>PROD-2026-1008</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="B31" t="str">
-        <v>Premium Industrial Product Variant 8</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="C31" t="str">
-        <v>Weight</v>
+        <v>Outer Diameter (D)</v>
       </c>
       <c r="D31" t="str">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="E31" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>PROD-2026-1008</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="B32" t="str">
-        <v>Premium Industrial Product Variant 8</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="C32" t="str">
-        <v>Warranty</v>
+        <v>Width (B)</v>
       </c>
       <c r="D32" t="str">
-        <v>2 Years</v>
+        <v>31</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>PROD-2026-1008</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="B33" t="str">
-        <v>Premium Industrial Product Variant 8</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="C33" t="str">
-        <v>Safety Standard</v>
+        <v>Dynamic Load Rating</v>
       </c>
       <c r="D33" t="str">
-        <v>ISO 9001:2015</v>
+        <v>85.2</v>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>kN</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>PROD-2026-1009</v>
+        <v>BRG-DGB-6312-2RS</v>
       </c>
       <c r="B34" t="str">
-        <v>Premium Industrial Product Variant 9</v>
+        <v>Deep Groove Ball Bearing 6312-2RS1/C3 (60x130x31 mm)</v>
       </c>
       <c r="C34" t="str">
-        <v>Material</v>
+        <v>Limiting Speed</v>
       </c>
       <c r="D34" t="str">
-        <v>High-Grade Alloy Type 9</v>
+        <v>3800</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>RPM</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>PROD-2026-1009</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="B35" t="str">
-        <v>Premium Industrial Product Variant 9</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="C35" t="str">
-        <v>Weight</v>
+        <v>Bore Diameter</v>
       </c>
       <c r="D35" t="str">
-        <v>13.5</v>
+        <v>100</v>
       </c>
       <c r="E35" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>PROD-2026-1009</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="B36" t="str">
-        <v>Premium Industrial Product Variant 9</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="C36" t="str">
-        <v>Warranty</v>
+        <v>Stroke Length</v>
       </c>
       <c r="D36" t="str">
-        <v>2 Years</v>
+        <v>400</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>PROD-2026-1009</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="B37" t="str">
-        <v>Premium Industrial Product Variant 9</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="C37" t="str">
-        <v>Safety Standard</v>
+        <v>Operating Pressure</v>
       </c>
       <c r="D37" t="str">
-        <v>ISO 9001:2015</v>
+        <v>210</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>Bar</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>PROD-2026-1010</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="B38" t="str">
-        <v>Premium Industrial Product Variant 10</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="C38" t="str">
-        <v>Material</v>
+        <v>Piston Rod Diameter</v>
       </c>
       <c r="D38" t="str">
-        <v>High-Grade Alloy Type 10</v>
+        <v>56</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>PROD-2026-1010</v>
+        <v>HYD-CYL-100-400</v>
       </c>
       <c r="B39" t="str">
-        <v>Premium Industrial Product Variant 10</v>
+        <v>Double-Acting Heavy Duty Industrial Hydraulic Cylinder (100mm Bore x 400mm Stroke)</v>
       </c>
       <c r="C39" t="str">
-        <v>Weight</v>
+        <v>Proof Pressure</v>
       </c>
       <c r="D39" t="str">
-        <v>15</v>
+        <v>315</v>
       </c>
       <c r="E39" t="str">
-        <v>Kg</v>
+        <v>Bar</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>PROD-2026-1010</v>
+        <v>CEM-PSC-50KG</v>
       </c>
       <c r="B40" t="str">
-        <v>Premium Industrial Product Variant 10</v>
+        <v>Portland Slag Cement (PSC) 50 Kg Moisture-Proof Bags</v>
       </c>
       <c r="C40" t="str">
-        <v>Warranty</v>
+        <v>Standard Conformance</v>
       </c>
       <c r="D40" t="str">
-        <v>2 Years</v>
+        <v>IS 455:2015</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -2648,203 +2648,203 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>PROD-2026-1010</v>
+        <v>CEM-PSC-50KG</v>
       </c>
       <c r="B41" t="str">
-        <v>Premium Industrial Product Variant 10</v>
+        <v>Portland Slag Cement (PSC) 50 Kg Moisture-Proof Bags</v>
       </c>
       <c r="C41" t="str">
-        <v>Safety Standard</v>
+        <v>Bag Weight</v>
       </c>
       <c r="D41" t="str">
-        <v>ISO 9001:2015</v>
+        <v>50</v>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>Kg</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>PROD-2026-1011</v>
+        <v>CEM-PSC-50KG</v>
       </c>
       <c r="B42" t="str">
-        <v>Premium Industrial Product Variant 11</v>
+        <v>Portland Slag Cement (PSC) 50 Kg Moisture-Proof Bags</v>
       </c>
       <c r="C42" t="str">
-        <v>Material</v>
+        <v>28-Day Compressive Strength</v>
       </c>
       <c r="D42" t="str">
-        <v>High-Grade Alloy Type 11</v>
+        <v>52</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>MPa</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>PROD-2026-1011</v>
+        <v>CEM-PSC-50KG</v>
       </c>
       <c r="B43" t="str">
-        <v>Premium Industrial Product Variant 11</v>
+        <v>Portland Slag Cement (PSC) 50 Kg Moisture-Proof Bags</v>
       </c>
       <c r="C43" t="str">
-        <v>Weight</v>
+        <v>Initial Setting Time</v>
       </c>
       <c r="D43" t="str">
-        <v>16.5</v>
+        <v>140</v>
       </c>
       <c r="E43" t="str">
-        <v>Kg</v>
+        <v>Minutes</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>PROD-2026-1011</v>
+        <v>WELD-INV-400A-3P</v>
       </c>
       <c r="B44" t="str">
-        <v>Premium Industrial Product Variant 11</v>
+        <v>IGBT Multi-Process Inverter Welding Machine (400 Amp, 3-Phase)</v>
       </c>
       <c r="C44" t="str">
-        <v>Warranty</v>
+        <v>Output Current Range</v>
       </c>
       <c r="D44" t="str">
-        <v>2 Years</v>
+        <v>20 - 400</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>Amps</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>PROD-2026-1011</v>
+        <v>WELD-INV-400A-3P</v>
       </c>
       <c r="B45" t="str">
-        <v>Premium Industrial Product Variant 11</v>
+        <v>IGBT Multi-Process Inverter Welding Machine (400 Amp, 3-Phase)</v>
       </c>
       <c r="C45" t="str">
-        <v>Safety Standard</v>
+        <v>Input Voltage</v>
       </c>
       <c r="D45" t="str">
-        <v>ISO 9001:2015</v>
+        <v>415V ± 15% (3-Phase)</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>V</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>PROD-2026-1012</v>
+        <v>WELD-INV-400A-3P</v>
       </c>
       <c r="B46" t="str">
-        <v>Premium Industrial Product Variant 12</v>
+        <v>IGBT Multi-Process Inverter Welding Machine (400 Amp, 3-Phase)</v>
       </c>
       <c r="C46" t="str">
-        <v>Material</v>
+        <v>Duty Cycle at 400A</v>
       </c>
       <c r="D46" t="str">
-        <v>High-Grade Alloy Type 12</v>
+        <v>60</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>%</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>PROD-2026-1012</v>
+        <v>WELD-INV-400A-3P</v>
       </c>
       <c r="B47" t="str">
-        <v>Premium Industrial Product Variant 12</v>
+        <v>IGBT Multi-Process Inverter Welding Machine (400 Amp, 3-Phase)</v>
       </c>
       <c r="C47" t="str">
-        <v>Weight</v>
+        <v>Usable Electrode Diameter</v>
       </c>
       <c r="D47" t="str">
-        <v>18</v>
+        <v>2.5 - 5.0</v>
       </c>
       <c r="E47" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>PROD-2026-1012</v>
+        <v>REF-BRK-HA70-IS8</v>
       </c>
       <c r="B48" t="str">
-        <v>Premium Industrial Product Variant 12</v>
+        <v>High Alumina 70% Industrial Refractory Fire Bricks (IS 8 Standard)</v>
       </c>
       <c r="C48" t="str">
-        <v>Warranty</v>
+        <v>Alumina Content (Al2O3)</v>
       </c>
       <c r="D48" t="str">
-        <v>2 Years</v>
+        <v>70</v>
       </c>
       <c r="E48" t="str">
-        <v/>
+        <v>%</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>PROD-2026-1012</v>
+        <v>REF-BRK-HA70-IS8</v>
       </c>
       <c r="B49" t="str">
-        <v>Premium Industrial Product Variant 12</v>
+        <v>High Alumina 70% Industrial Refractory Fire Bricks (IS 8 Standard)</v>
       </c>
       <c r="C49" t="str">
-        <v>Safety Standard</v>
+        <v>Refractoriness (PCE)</v>
       </c>
       <c r="D49" t="str">
-        <v>ISO 9001:2015</v>
+        <v>+37 (&gt; 1820°C)</v>
       </c>
       <c r="E49" t="str">
-        <v/>
+        <v>PCE</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>PROD-2026-1013</v>
+        <v>REF-BRK-HA70-IS8</v>
       </c>
       <c r="B50" t="str">
-        <v>Premium Industrial Product Variant 13</v>
+        <v>High Alumina 70% Industrial Refractory Fire Bricks (IS 8 Standard)</v>
       </c>
       <c r="C50" t="str">
-        <v>Material</v>
+        <v>Bulk Density</v>
       </c>
       <c r="D50" t="str">
-        <v>High-Grade Alloy Type 13</v>
+        <v>2.68</v>
       </c>
       <c r="E50" t="str">
-        <v/>
+        <v>g/cc</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>PROD-2026-1013</v>
+        <v>REF-BRK-HA70-IS8</v>
       </c>
       <c r="B51" t="str">
-        <v>Premium Industrial Product Variant 13</v>
+        <v>High Alumina 70% Industrial Refractory Fire Bricks (IS 8 Standard)</v>
       </c>
       <c r="C51" t="str">
-        <v>Weight</v>
+        <v>Cold Crushing Strength</v>
       </c>
       <c r="D51" t="str">
-        <v>19.5</v>
+        <v>650</v>
       </c>
       <c r="E51" t="str">
-        <v>Kg</v>
+        <v>kg/cm²</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>PROD-2026-1013</v>
+        <v>SHG-SAM-SAREE-01</v>
       </c>
       <c r="B52" t="str">
-        <v>Premium Industrial Product Variant 13</v>
+        <v>Authentic Sambalpuri Handloom Pure Cotton Ikat Saree (GI Certified)</v>
       </c>
       <c r="C52" t="str">
-        <v>Warranty</v>
+        <v>Fabric</v>
       </c>
       <c r="D52" t="str">
-        <v>2 Years</v>
+        <v>100% Pure Organic Combed Cotton</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -2852,16 +2852,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>PROD-2026-1013</v>
+        <v>SHG-SAM-SAREE-01</v>
       </c>
       <c r="B53" t="str">
-        <v>Premium Industrial Product Variant 13</v>
+        <v>Authentic Sambalpuri Handloom Pure Cotton Ikat Saree (GI Certified)</v>
       </c>
       <c r="C53" t="str">
-        <v>Safety Standard</v>
+        <v>Weave Pattern</v>
       </c>
       <c r="D53" t="str">
-        <v>ISO 9001:2015</v>
+        <v>Traditional Odisha Bandhakala (Ikat)</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -2869,50 +2869,50 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>PROD-2026-1014</v>
+        <v>SHG-SAM-SAREE-01</v>
       </c>
       <c r="B54" t="str">
-        <v>Premium Industrial Product Variant 14</v>
+        <v>Authentic Sambalpuri Handloom Pure Cotton Ikat Saree (GI Certified)</v>
       </c>
       <c r="C54" t="str">
-        <v>Material</v>
+        <v>Saree Length</v>
       </c>
       <c r="D54" t="str">
-        <v>High-Grade Alloy Type 14</v>
+        <v>6.3 (with Blouse Piece)</v>
       </c>
       <c r="E54" t="str">
-        <v/>
+        <v>Meters</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>PROD-2026-1014</v>
+        <v>SHG-SAM-SAREE-01</v>
       </c>
       <c r="B55" t="str">
-        <v>Premium Industrial Product Variant 14</v>
+        <v>Authentic Sambalpuri Handloom Pure Cotton Ikat Saree (GI Certified)</v>
       </c>
       <c r="C55" t="str">
-        <v>Weight</v>
+        <v>Origin Certification</v>
       </c>
       <c r="D55" t="str">
-        <v>21</v>
+        <v>Geographical Indication (GI) Tagged</v>
       </c>
       <c r="E55" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>PROD-2026-1014</v>
+        <v>SHG-DHK-FIG-08</v>
       </c>
       <c r="B56" t="str">
-        <v>Premium Industrial Product Variant 14</v>
+        <v>Odisha Dhokra Brass Lost-Wax Casting Tribal Art Figurine (8-Inch)</v>
       </c>
       <c r="C56" t="str">
-        <v>Warranty</v>
+        <v>Material</v>
       </c>
       <c r="D56" t="str">
-        <v>2 Years</v>
+        <v>Brass / Bronze Bell Metal Alloy</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -2920,67 +2920,67 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>PROD-2026-1014</v>
+        <v>SHG-DHK-FIG-08</v>
       </c>
       <c r="B57" t="str">
-        <v>Premium Industrial Product Variant 14</v>
+        <v>Odisha Dhokra Brass Lost-Wax Casting Tribal Art Figurine (8-Inch)</v>
       </c>
       <c r="C57" t="str">
-        <v>Safety Standard</v>
+        <v>Height</v>
       </c>
       <c r="D57" t="str">
-        <v>ISO 9001:2015</v>
+        <v>8</v>
       </c>
       <c r="E57" t="str">
-        <v/>
+        <v>Inch</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>PROD-2026-1015</v>
+        <v>SHG-DHK-FIG-08</v>
       </c>
       <c r="B58" t="str">
-        <v>Premium Industrial Product Variant 15</v>
+        <v>Odisha Dhokra Brass Lost-Wax Casting Tribal Art Figurine (8-Inch)</v>
       </c>
       <c r="C58" t="str">
-        <v>Material</v>
+        <v>Weight</v>
       </c>
       <c r="D58" t="str">
-        <v>High-Grade Alloy Type 15</v>
+        <v>1.1</v>
       </c>
       <c r="E58" t="str">
-        <v/>
+        <v>Kg</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>PROD-2026-1015</v>
+        <v>SHG-DHK-FIG-08</v>
       </c>
       <c r="B59" t="str">
-        <v>Premium Industrial Product Variant 15</v>
+        <v>Odisha Dhokra Brass Lost-Wax Casting Tribal Art Figurine (8-Inch)</v>
       </c>
       <c r="C59" t="str">
-        <v>Weight</v>
+        <v>Craft Technique</v>
       </c>
       <c r="D59" t="str">
-        <v>22.5</v>
+        <v>Lost Wax Metal Casting (Cire Perdue)</v>
       </c>
       <c r="E59" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>PROD-2026-1015</v>
+        <v>SAF-GLV-NIT-15</v>
       </c>
       <c r="B60" t="str">
-        <v>Premium Industrial Product Variant 15</v>
+        <v>Industrial Heavy Duty Nitrile Chemical Gauntlet Gloves (15-Inch, 15 Mil)</v>
       </c>
       <c r="C60" t="str">
-        <v>Warranty</v>
+        <v>Material</v>
       </c>
       <c r="D60" t="str">
-        <v>2 Years</v>
+        <v>100% Acrylonitrile Butadiene</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -2988,220 +2988,220 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>PROD-2026-1015</v>
+        <v>SAF-GLV-NIT-15</v>
       </c>
       <c r="B61" t="str">
-        <v>Premium Industrial Product Variant 15</v>
+        <v>Industrial Heavy Duty Nitrile Chemical Gauntlet Gloves (15-Inch, 15 Mil)</v>
       </c>
       <c r="C61" t="str">
-        <v>Safety Standard</v>
+        <v>Glove Length</v>
       </c>
       <c r="D61" t="str">
-        <v>ISO 9001:2015</v>
+        <v>15 (380mm)</v>
       </c>
       <c r="E61" t="str">
-        <v/>
+        <v>Inch</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>PROD-2026-1016</v>
+        <v>SAF-GLV-NIT-15</v>
       </c>
       <c r="B62" t="str">
-        <v>Premium Industrial Product Variant 16</v>
+        <v>Industrial Heavy Duty Nitrile Chemical Gauntlet Gloves (15-Inch, 15 Mil)</v>
       </c>
       <c r="C62" t="str">
-        <v>Material</v>
+        <v>Thickness</v>
       </c>
       <c r="D62" t="str">
-        <v>High-Grade Alloy Type 16</v>
+        <v>15</v>
       </c>
       <c r="E62" t="str">
-        <v/>
+        <v>Mil</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>PROD-2026-1016</v>
+        <v>SAF-GLV-NIT-15</v>
       </c>
       <c r="B63" t="str">
-        <v>Premium Industrial Product Variant 16</v>
+        <v>Industrial Heavy Duty Nitrile Chemical Gauntlet Gloves (15-Inch, 15 Mil)</v>
       </c>
       <c r="C63" t="str">
-        <v>Weight</v>
+        <v>Standard Rating</v>
       </c>
       <c r="D63" t="str">
-        <v>24</v>
+        <v>EN 388 (4101X) / EN ISO 374-1 Type A</v>
       </c>
       <c r="E63" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>PROD-2026-1016</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="B64" t="str">
-        <v>Premium Industrial Product Variant 16</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="C64" t="str">
-        <v>Warranty</v>
+        <v>Belt Width</v>
       </c>
       <c r="D64" t="str">
-        <v>2 Years</v>
+        <v>800</v>
       </c>
       <c r="E64" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>PROD-2026-1016</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="B65" t="str">
-        <v>Premium Industrial Product Variant 16</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="C65" t="str">
-        <v>Safety Standard</v>
+        <v>Tensile Strength</v>
       </c>
       <c r="D65" t="str">
-        <v>ISO 9001:2015</v>
+        <v>400</v>
       </c>
       <c r="E65" t="str">
-        <v/>
+        <v>N/mm</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>PROD-2026-1017</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="B66" t="str">
-        <v>Premium Industrial Product Variant 17</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="C66" t="str">
-        <v>Material</v>
+        <v>Number of Plies</v>
       </c>
       <c r="D66" t="str">
-        <v>High-Grade Alloy Type 17</v>
+        <v>3</v>
       </c>
       <c r="E66" t="str">
-        <v/>
+        <v>Plies</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>PROD-2026-1017</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="B67" t="str">
-        <v>Premium Industrial Product Variant 17</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="C67" t="str">
-        <v>Weight</v>
+        <v>Temperature Rating</v>
       </c>
       <c r="D67" t="str">
-        <v>25.5</v>
+        <v>Up to 150°C continuous</v>
       </c>
       <c r="E67" t="str">
-        <v>Kg</v>
+        <v>°C</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PROD-2026-1017</v>
+        <v>CNV-BLT-EP400-800</v>
       </c>
       <c r="B68" t="str">
-        <v>Premium Industrial Product Variant 17</v>
+        <v>Heat-Resistant EP Rubber Conveyor Belt (EP 400/3, 800mm Wide)</v>
       </c>
       <c r="C68" t="str">
-        <v>Warranty</v>
+        <v>Top / Bottom Rubber Cover</v>
       </c>
       <c r="D68" t="str">
-        <v>2 Years</v>
+        <v>5mm / 2mm Grade HR</v>
       </c>
       <c r="E68" t="str">
-        <v/>
+        <v>mm</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>PROD-2026-1017</v>
+        <v>CHM-CS-FLK-50KG</v>
       </c>
       <c r="B69" t="str">
-        <v>Premium Industrial Product Variant 17</v>
+        <v>Technical Grade Caustic Soda Flakes / Sodium Hydroxide (99.5% Pure, 50kg)</v>
       </c>
       <c r="C69" t="str">
-        <v>Safety Standard</v>
+        <v>Assay (as NaOH)</v>
       </c>
       <c r="D69" t="str">
-        <v>ISO 9001:2015</v>
+        <v>99.5 Min</v>
       </c>
       <c r="E69" t="str">
-        <v/>
+        <v>%</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>PROD-2026-1018</v>
+        <v>CHM-CS-FLK-50KG</v>
       </c>
       <c r="B70" t="str">
-        <v>Premium Industrial Product Variant 18</v>
+        <v>Technical Grade Caustic Soda Flakes / Sodium Hydroxide (99.5% Pure, 50kg)</v>
       </c>
       <c r="C70" t="str">
-        <v>Material</v>
+        <v>Sodium Carbonate (Na2CO3)</v>
       </c>
       <c r="D70" t="str">
-        <v>High-Grade Alloy Type 18</v>
+        <v>0.4 Max</v>
       </c>
       <c r="E70" t="str">
-        <v/>
+        <v>%</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>PROD-2026-1018</v>
+        <v>CHM-CS-FLK-50KG</v>
       </c>
       <c r="B71" t="str">
-        <v>Premium Industrial Product Variant 18</v>
+        <v>Technical Grade Caustic Soda Flakes / Sodium Hydroxide (99.5% Pure, 50kg)</v>
       </c>
       <c r="C71" t="str">
-        <v>Weight</v>
+        <v>Form</v>
       </c>
       <c r="D71" t="str">
-        <v>27</v>
+        <v>Dry White Deliquescent Flakes</v>
       </c>
       <c r="E71" t="str">
-        <v>Kg</v>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>PROD-2026-1018</v>
+        <v>CHM-CS-FLK-50KG</v>
       </c>
       <c r="B72" t="str">
-        <v>Premium Industrial Product Variant 18</v>
+        <v>Technical Grade Caustic Soda Flakes / Sodium Hydroxide (99.5% Pure, 50kg)</v>
       </c>
       <c r="C72" t="str">
-        <v>Warranty</v>
+        <v>Packaging</v>
       </c>
       <c r="D72" t="str">
-        <v>2 Years</v>
+        <v>50 Kg HDPE Laminated Bags with Liner</v>
       </c>
       <c r="E72" t="str">
-        <v/>
+        <v>Kg</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>PROD-2026-1018</v>
+        <v>TYR-R20-16PR-HD</v>
       </c>
       <c r="B73" t="str">
-        <v>Premium Industrial Product Variant 18</v>
+        <v>Heavy Duty Mining Dumper Radial Tyre (10.00 R20 16PR All-Steel)</v>
       </c>
       <c r="C73" t="str">
-        <v>Safety Standard</v>
+        <v>Tyre Size</v>
       </c>
       <c r="D73" t="str">
-        <v>ISO 9001:2015</v>
+        <v>10.00 R20</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -3209,50 +3209,50 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>PROD-2026-1019</v>
+        <v>TYR-R20-16PR-HD</v>
       </c>
       <c r="B74" t="str">
-        <v>Premium Industrial Product Variant 19</v>
+        <v>Heavy Duty Mining Dumper Radial Tyre (10.00 R20 16PR All-Steel)</v>
       </c>
       <c r="C74" t="str">
-        <v>Material</v>
+        <v>Ply Rating</v>
       </c>
       <c r="D74" t="str">
-        <v>High-Grade Alloy Type 19</v>
+        <v>16</v>
       </c>
       <c r="E74" t="str">
-        <v/>
+        <v>PR</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>PROD-2026-1019</v>
+        <v>TYR-R20-16PR-HD</v>
       </c>
       <c r="B75" t="str">
-        <v>Premium Industrial Product Variant 19</v>
+        <v>Heavy Duty Mining Dumper Radial Tyre (10.00 R20 16PR All-Steel)</v>
       </c>
       <c r="C75" t="str">
-        <v>Weight</v>
+        <v>Tread Depth</v>
       </c>
       <c r="D75" t="str">
-        <v>28.5</v>
+        <v>16.5</v>
       </c>
       <c r="E75" t="str">
-        <v>Kg</v>
+        <v>mm</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>PROD-2026-1019</v>
+        <v>TYR-R20-16PR-HD</v>
       </c>
       <c r="B76" t="str">
-        <v>Premium Industrial Product Variant 19</v>
+        <v>Heavy Duty Mining Dumper Radial Tyre (10.00 R20 16PR All-Steel)</v>
       </c>
       <c r="C76" t="str">
-        <v>Warranty</v>
+        <v>Speed Symbol / Load Index</v>
       </c>
       <c r="D76" t="str">
-        <v>2 Years</v>
+        <v>146/143 K (3000 kg/tyre)</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -3260,16 +3260,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>PROD-2026-1019</v>
+        <v>IT-SRV-2U-XEON-64</v>
       </c>
       <c r="B77" t="str">
-        <v>Premium Industrial Product Variant 19</v>
+        <v>Enterprise 2U Rackmount Server Dual Intel Xeon Silver 64GB ECC RAM</v>
       </c>
       <c r="C77" t="str">
-        <v>Safety Standard</v>
+        <v>Processor</v>
       </c>
       <c r="D77" t="str">
-        <v>ISO 9001:2015</v>
+        <v>2x Intel Xeon Silver 4310 (24 Cores total)</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -3277,50 +3277,50 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>PROD-2026-1020</v>
+        <v>IT-SRV-2U-XEON-64</v>
       </c>
       <c r="B78" t="str">
-        <v>Premium Industrial Product Variant 20</v>
+        <v>Enterprise 2U Rackmount Server Dual Intel Xeon Silver 64GB ECC RAM</v>
       </c>
       <c r="C78" t="str">
-        <v>Material</v>
+        <v>Memory</v>
       </c>
       <c r="D78" t="str">
-        <v>High-Grade Alloy Type 20</v>
+        <v>64GB (2x32GB) DDR4-3200 ECC RDIMM</v>
       </c>
       <c r="E78" t="str">
-        <v/>
+        <v>GB</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>PROD-2026-1020</v>
+        <v>IT-SRV-2U-XEON-64</v>
       </c>
       <c r="B79" t="str">
-        <v>Premium Industrial Product Variant 20</v>
+        <v>Enterprise 2U Rackmount Server Dual Intel Xeon Silver 64GB ECC RAM</v>
       </c>
       <c r="C79" t="str">
-        <v>Weight</v>
+        <v>Storage</v>
       </c>
       <c r="D79" t="str">
-        <v>30</v>
+        <v>2x 960GB Enterprise SAS Mixed-Use SSD</v>
       </c>
       <c r="E79" t="str">
-        <v>Kg</v>
+        <v>GB</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>PROD-2026-1020</v>
+        <v>IT-SRV-2U-XEON-64</v>
       </c>
       <c r="B80" t="str">
-        <v>Premium Industrial Product Variant 20</v>
+        <v>Enterprise 2U Rackmount Server Dual Intel Xeon Silver 64GB ECC RAM</v>
       </c>
       <c r="C80" t="str">
-        <v>Warranty</v>
+        <v>RAID Controller</v>
       </c>
       <c r="D80" t="str">
-        <v>2 Years</v>
+        <v>Hardware PERC H745 with 4GB NV Cache</v>
       </c>
       <c r="E80" t="str">
         <v/>
@@ -3328,24 +3328,143 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>PROD-2026-1020</v>
+        <v>TOOL-AIW-1IN-2600</v>
       </c>
       <c r="B81" t="str">
-        <v>Premium Industrial Product Variant 20</v>
+        <v>Pneumatic Heavy Duty Industrial Air Impact Wrench (1-Inch Drive, 2600 Nm)</v>
       </c>
       <c r="C81" t="str">
-        <v>Safety Standard</v>
+        <v>Square Drive Size</v>
       </c>
       <c r="D81" t="str">
-        <v>ISO 9001:2015</v>
+        <v>1</v>
       </c>
       <c r="E81" t="str">
+        <v>Inch</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>TOOL-AIW-1IN-2600</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Pneumatic Heavy Duty Industrial Air Impact Wrench (1-Inch Drive, 2600 Nm)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Max Working Torque</v>
+      </c>
+      <c r="D82" t="str">
+        <v>2600</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Nm</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>TOOL-AIW-1IN-2600</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Pneumatic Heavy Duty Industrial Air Impact Wrench (1-Inch Drive, 2600 Nm)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Free Speed</v>
+      </c>
+      <c r="D83" t="str">
+        <v>4200</v>
+      </c>
+      <c r="E83" t="str">
+        <v>RPM</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>TOOL-AIW-1IN-2600</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Pneumatic Heavy Duty Industrial Air Impact Wrench (1-Inch Drive, 2600 Nm)</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Recommended Air Pressure</v>
+      </c>
+      <c r="D84" t="str">
+        <v>6.2 - 8.0</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Bar</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>AUTO-PLC-PNL-7HMI</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Industrial PLC Automation Control Panel with 7-Inch Color Touch HMI</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Main Controller</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Siemens Simatic S7-1200 CPU 1214C DC/DC/DC</v>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>AUTO-PLC-PNL-7HMI</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Industrial PLC Automation Control Panel with 7-Inch Color Touch HMI</v>
+      </c>
+      <c r="C86" t="str">
+        <v>HMI Touch Display</v>
+      </c>
+      <c r="D86" t="str">
+        <v>7 Inch 800x480 Widescreen 65K Colors</v>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>AUTO-PLC-PNL-7HMI</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Industrial PLC Automation Control Panel with 7-Inch Color Touch HMI</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Communication Protocol</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Profinet / Modbus TCP/IP</v>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>AUTO-PLC-PNL-7HMI</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Industrial PLC Automation Control Panel with 7-Inch Color Touch HMI</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Enclosure Protection</v>
+      </c>
+      <c r="D88" t="str">
+        <v>IP65 Powder Coated CRCA Steel 2mm</v>
+      </c>
+      <c r="E88" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E88"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3361,47 +3480,47 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tyres &amp; Rubber Products</v>
+        <v>Agriculture &amp; Nursery</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Fuel, Oil &amp; Gas</v>
+        <v>Automation &amp; Robotics</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Power &amp; Energy Equipment</v>
+        <v>Automobile Parts &amp; Services</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Refractories</v>
+        <v>Bearings &amp; Mechanical Components</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Automobile Parts &amp; Services</v>
+        <v>Cement &amp; Concrete Products</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Office Equipment &amp; Stationery</v>
+        <v>Construction &amp; Building Materials</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Bearings &amp; Mechanical Components</v>
+        <v>Conveyor &amp; Material Handling Equipment</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Construction &amp; Building Materials</v>
+        <v>Electrical &amp; Electronics</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Steel &amp; Metal Products</v>
+        <v>Electrical Cables &amp; Power Equipment</v>
       </c>
     </row>
     <row r="11">
@@ -3411,52 +3530,52 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>teeeeeee</v>
+        <v>Fuel, Oil &amp; Gas</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Industrial Chemicals</v>
+        <v>Furniture &amp; Interior Supplies</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Electrical Cables &amp; Power Equipment</v>
+        <v>Gas Equipment &amp; Cylinders</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Industrial Consumables</v>
+        <v>General Industrial Supplier</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>IT &amp; Computer Equipment</v>
+        <v>Hydraulics &amp; Pneumatics</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Tools &amp; Industrial Hardware</v>
+        <v>IT &amp; Computer Equipment</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Furniture &amp; Interior Supplies</v>
+        <v>Industrial Chemicals</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>General Industrial Supplier</v>
+        <v>Industrial Consumables</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Gas Equipment &amp; Cylinders</v>
+        <v>Industrial Fasteners &amp; Components</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Agriculture &amp; Nursery</v>
+        <v>Industrial Machinery &amp; Spare Parts</v>
       </c>
     </row>
     <row r="22">
@@ -3466,7 +3585,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Industrial Fasteners &amp; Components</v>
+        <v>Laboratory Equipment &amp; Chemicals</v>
       </c>
     </row>
     <row r="24">
@@ -3481,7 +3600,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Pumps, Motors &amp; Hydraulics</v>
+        <v>Mining &amp; Coal Equipment</v>
       </c>
     </row>
     <row r="27">
@@ -3491,12 +3610,12 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Electrical &amp; Electronics</v>
+        <v>OEM / Manufacturing Vendor</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Pipes, Tiles &amp; Hardware</v>
+        <v>Office Equipment &amp; Stationery</v>
       </c>
     </row>
     <row r="30">
@@ -3506,42 +3625,42 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Safety Equipment &amp; Industrial Safety</v>
+        <v>Pipes, Tiles &amp; Hardware</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Cement &amp; Concrete Products</v>
+        <v>Polymer &amp; Plastic Products</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Textile &amp; Garments Supply</v>
+        <v>Power &amp; Energy Equipment</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>OEM / Manufacturing Vendor</v>
+        <v>Pumps, Motors &amp; Hydraulics</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Industrial Machinery &amp; Spare Parts</v>
+        <v>Refractories</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Automation &amp; Robotics</v>
+        <v>Retail &amp; Commercial Supply</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Polymer &amp; Plastic Products</v>
+        <v>Safety Equipment &amp; Industrial Safety</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Laboratory Equipment &amp; Chemicals</v>
+        <v>Steel &amp; Metal Products</v>
       </c>
     </row>
     <row r="39">
@@ -3551,27 +3670,27 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Mining &amp; Coal Equipment</v>
+        <v>Textile &amp; Garments Supply</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Hydraulics &amp; Pneumatics</v>
+        <v>Tools &amp; Industrial Hardware</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Welding &amp; Cutting Equipment</v>
+        <v>Tyres &amp; Rubber Products</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Retail &amp; Commercial Supply</v>
+        <v>Welding &amp; Cutting Equipment</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Conveyor &amp; Material Handling Equipment</v>
+        <v>test 1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add seed template generator and implementation for catalogue import service
</commit_message>
<xml_diff>
--- a/backend/seeded_templates/Seeded_Products_Import.xlsx
+++ b/backend/seeded_templates/Seeded_Products_Import.xlsx
@@ -546,7 +546,7 @@
         <v>https://images.unsplash.com/photo-1618090584176-7132b9911657?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X2" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="3">
@@ -694,7 +694,7 @@
         <v>https://images.unsplash.com/photo-1565043666747-69f6646db940?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X4" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="5">
@@ -842,7 +842,7 @@
         <v>https://images.unsplash.com/photo-1621905251189-08b45d6a269e?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X6" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="7">
@@ -913,7 +913,7 @@
         <v>500</v>
       </c>
       <c r="W7" t="str">
-        <v>https://images.unsplash.com/photo-1581092795360-fd1ca04f0952?w=1200&amp;auto=format&amp;fit=crop</v>
+        <v>https://images.unsplash.com/photo-1586864387967-d02ef85d93e8?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X7" t="str">
         <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/web/compressed.tracemonkey-pldi-09.pdf</v>
@@ -990,7 +990,7 @@
         <v>https://images.unsplash.com/photo-1581092334651-ddf26d9a09d0?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X8" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="9">
@@ -1138,7 +1138,7 @@
         <v>https://images.unsplash.com/photo-1587293852726-70cdb56c2866?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X10" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="11">
@@ -1286,7 +1286,7 @@
         <v>https://images.unsplash.com/photo-1587293852726-70cdb56c2866?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X12" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="13">
@@ -1434,7 +1434,7 @@
         <v>https://images.unsplash.com/photo-1590736704728-f4730bb30770?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X14" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="15">
@@ -1582,7 +1582,7 @@
         <v>https://images.unsplash.com/photo-1586528116311-ad8dd3c8310d?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X16" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="17">
@@ -1730,7 +1730,7 @@
         <v>https://images.unsplash.com/photo-1517524008697-84bbe3c3fd98?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X18" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="19">
@@ -1878,7 +1878,7 @@
         <v>https://images.unsplash.com/photo-1530124566582-a618bc2615dc?w=1200&amp;auto=format&amp;fit=crop</v>
       </c>
       <c r="X20" t="str">
-        <v>https://www.w3.org/WAI/ER/tests/xhtml/testfiles/resources/pdf/dummy.pdf</v>
+        <v>https://raw.githubusercontent.com/mozilla/pdf.js/ba2edeae/test/pdfs/basicapi.pdf</v>
       </c>
     </row>
     <row r="21">

</xml_diff>